<commit_message>
Write AI and literacy syllabi into the school sheet tabs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P2HwXKeAyjzNfZEc1H8N6T
</commit_message>
<xml_diff>
--- a/docs/drafts/syllabus-sheets/syllabus.xlsx
+++ b/docs/drafts/syllabus-sheets/syllabus.xlsx
@@ -1676,10 +1676,10 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>日本語で書かれたルールを読み、張り紙・スライド・表・画像を作る。
-AIの答えはそのまま使わず、原文と比べて誤りを自分で直す。
-依頼を受けてから届けるまでを一人で行う。回が進むと材料と条件が増える。
-わからない時はAIで自分で解決する。マーケティング・ビジネス情報リテラシーにつながる。</t>
+          <t>架空の学校の図書室や事務室から「利用ルールの張り紙を作り、利用記録を集計してほしい」と頼まれた設定で進める。
+先輩がAIで作った下書きをルールの原文だけを正として直し、張り紙（Googleドキュメント）・Googleスライド・集計表（スプレッドシート）・画像の4つを作る。
+作ったものは共有設定とGoogleフォームで提出する。回が進むとGmailでの納品やGoogleカレンダーの招待が加わる。
+わからない時はGeminiで自分で解決し、出てきた答えや式は必ず確かめる。</t>
         </is>
       </c>
       <c r="B6" s="2" t="n"/>
@@ -1688,9 +1688,9 @@
       <c r="E6" s="5" t="inlineStr">
         <is>
           <t>基本教材：Geminiビジネス活用ガイド（最新の機能で扱う）
-教員が作った材料（ルールの原文・AIの下書き・利用記録）を毎回配る
+材料：教員が作ったルールの原文・AIの下書き・利用記録を毎回配る
 環境：スマホ、個人の Google アカウント（無料）
-ツール：Gemini、Gemini Notebook、画像生成、スプレッドシート、スライド、ドキュメント、ドライブ、Gmail、カレンダー、Meet、クラスルーム</t>
+ツール：Gemini、Gemini Notebook、ドキュメント、スライド、スプレッドシート、ドライブ、フォト、フォーム、Gmail、カレンダー、Meet</t>
         </is>
       </c>
       <c r="F6" s="2" t="n"/>
@@ -1758,10 +1758,10 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>1. 原文だけを正として、AIの下書きの誤りを直せる。
-2. AIに作らせた式の結果を確かめ、集計表を作れる。
-3. 条件を守った画像を3枚そろえ、約束どおりのスライドを作れる。
-4. 作ったものをメール・共有・予定の招待で届けられる。</t>
+          <t>1. ルールの原文だけを正として、AIの下書きの誤りを直した張り紙と誤り一覧を作成できる。
+2. Geminiに作らせた式を検算し、行を足しても正しく動く集計表をスプレッドシートで作成できる。
+3. 条件を守った画像を3枚そろえ、約束どおりの形のGoogleスライドを作成できる。
+4. 作ったものを共有設定・Gmail・Googleカレンダーの招待で届けられる。</t>
         </is>
       </c>
       <c r="B12" s="2" t="n"/>
@@ -1770,13 +1770,8 @@
       <c r="E12" s="5" t="inlineStr">
         <is>
           <t>採点基準は学校規定に準ずる。
-【独自の基準】
-・成果物は、課題ごとに示した条件を1つずつ○✖で見て、○の分だけ点を足す。1か所まちがえても、ほかの点は失わない。
-・本人が作った証拠（合言葉・画面録画・版の履歴など）が無い提出は0点。
-・材料の数字は学生ごとに違う。他人の答えを写しても点にならない。
-・作業時間は目安で、採点しない。受付時間はクラスルームで課題ごとに設定する。
-・小テストは満点で○。点＝20×○の数÷13（成果物の回は行わない）。欠席は✖。
-・出席率70%の学生でも、成果物で48点取ればD（60点）に届く設計にしている。</t>
+成果物は、課題ごとの条件を満たした分だけ点を足す。
+本人が作った証拠（録画など）の無い提出は0点。</t>
         </is>
       </c>
       <c r="F12" s="2" t="n"/>
@@ -1844,8 +1839,8 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>成果物 80点（8・12・15・20・25点）
-小テスト 20点（成果物の回を除く13回。満点まで再提出可）</t>
+          <t>成果物 80点（5回：8・12・15・20・25点）
+小テスト 20点（成果物の回以外の毎回）</t>
         </is>
       </c>
       <c r="B18" s="2" t="n"/>
@@ -1853,8 +1848,8 @@
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>小テスト：その場で結果を返し、満点まで再提出できる。
-成果物：本番の次の回に答え合わせをする（5・9・13・16回）。</t>
+          <t>小テストはその場で返し、満点まで出し直せる。
+成果物は前の回に練習し、本番の後に答え合わせをする。</t>
         </is>
       </c>
       <c r="F18" s="2" t="n"/>
@@ -1965,20 +1960,20 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>ガイダンス・ファイルの提出
+          <t>ガイダンス・共有と提出
 基本教材 2章1</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>作ったファイルを教員に届く形で提出できる。</t>
+          <t>ファイル名に合言葉を入れ、教員を編集者として共有し、Googleフォームで提出できる。</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>科目の進め方と評価。
-ファイル名と合言葉、教員への共有。
-Gemini Notebook に文章を貼る。</t>
+          <t>科目の進め方と評価。Geminiの基本操作。
+Googleドライブのファイル名と合言葉、共有設定（閲覧者/編集者）。
+Gemini Notebookに文章を貼る。</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -2006,19 +2001,20 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>原文を正として張り紙を直す
+          <t>原文と照合して張り紙を直す
 基本教材 5章1</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>原文だけを正として下書きを直せる。</t>
+          <t>Gemini Notebookで原文との照合表を作成し、下書きの誤りをGoogleドキュメントで直せる。</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Gemini Notebook で原文だけを根拠に答えさせる。
-照合表を作り、張り紙を直す。</t>
+          <t>Gemini Notebookで原文だけを根拠に答えさせる。
+照合表を作り、実在する語の誤字を探す。
+Googleドキュメントで張り紙を直す。</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -2046,19 +2042,19 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>式で数える・画像の画風
+          <t>式で数える・画風を変える
 基本教材 3章5・2章6</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>AIの式で数え、保つ点を守って画像を作れる。</t>
+          <t>Geminiの式で遅れの回数を数えて検算し、画風を変えた画像とGoogleスライド1枚を作成できる。</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>AIに式を作らせ、結果を確かめる。
-画像生成で画風を変える。スライド1枚。
+          <t>Geminiに式を作らせ、スプレッドシートで検算。
+画像生成で画風を変え、保つ点を守る。
 成果物1の通し練習（30分）。</t>
         </is>
       </c>
@@ -2087,12 +2083,12 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>成果物1　4つを一人で通す（実技）</t>
+          <t>成果物1　タブレット貸出しの張り紙一式（実技）</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>張り紙・スライド・集計表・画像を作って提出できる。</t>
+          <t>図書室の貸出しルールをもとに、張り紙・スライド1枚・集計表・画像を作成して提出できる。</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -2102,7 +2098,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>成果物1（クラスルーム）</t>
+          <t>成果物1</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -2117,7 +2113,7 @@
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>受付はクラスルームで設定。本人の証拠は合言葉と作成時刻</t>
+          <t>受付はクラスルームで設定</t>
         </is>
       </c>
     </row>
@@ -2135,13 +2131,14 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>下書きの誤りを数を知らされずに探し切れる。</t>
+          <t>Gemini Notebookで照合表を作成し、意味が違う誤字まで数を知らされずに探し切れる。</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
           <t>成果物1の答え合わせ。
-6件の照合、意味が違う誤字の練習。</t>
+Gemini Notebookで6件を照合。
+読めるのに意味が違う誤字を探す。</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -2175,13 +2172,13 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>出力を約束どおりの形に直し、上限ちょうどを正しく数えられる。</t>
+          <t>形の約束どおりのGoogleスライドを作成し、上限ちょうどを違反にしない式を検算できる。</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>出力の形を指示して文章を作る。
-「上限ちょうどは違反でない」式をAIに作らせ、確かめる。</t>
+          <t>Geminiに出力の形を指定する（枚数・右下の番号・括弧）。
+「上限ちょうどは違反でない」式をGeminiに作らせ、検算する。</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -2215,12 +2212,12 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>同じ条件の画像を3枚そろえ、1枚ずつ確かめられる。</t>
+          <t>同じ指示で画像を3枚生成し、保つ点（数・色・位置・比率）を1枚ずつ確かめられる。</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>同じ指示で3枚作り、保つ点を確かめる。
+          <t>同じ指示で3枚生成し、保つ点を1枚ずつ○✖で確かめる。
 成果物2の通し練習（40分）。</t>
         </is>
       </c>
@@ -2249,12 +2246,12 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>成果物2　条件の増えた一連の仕事（実技）</t>
+          <t>成果物2　グループ学習室の張り紙一式（実技）</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>誤りを直し、スライド・集計表・画像3枚を提出できる。</t>
+          <t>下書きの誤り6件を直し、張り紙・スライド2枚・集計表・画像3枚を作成して提出できる。</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -2264,7 +2261,7 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>成果物2（クラスルーム）</t>
+          <t>成果物2</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
@@ -2279,7 +2276,7 @@
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>受付はクラスルームで設定。本人の証拠は合言葉と作成時刻</t>
+          <t>受付はクラスルームで設定</t>
         </is>
       </c>
     </row>
@@ -2291,19 +2288,20 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>古い値と逆の文を見抜く
+          <t>旧版の値と原文と逆の文
 基本教材 3章3</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>旧版の値と原文と逆の文を見抜き、誤り一覧を作れる。</t>
+          <t>改定の記録から旧版の値と原文と逆の文を見抜き、誤り一覧をスプレッドシートで作成できる。</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
           <t>成果物2の答え合わせ。
-改定の記録を読み、誤り一覧を作る。</t>
+改定の記録を読み、旧版の値・原文と逆の追加を探す。
+誤り一覧（どの文・どう違う・正しい内容）を作る。</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -2331,19 +2329,19 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>行を足しても正しい表
+          <t>行を足しても正しい集計表
 基本教材 3章5</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>延長と停止の開始日を出し、行を足して確かめられる。</t>
+          <t>延長と予約停止の開始日を出す式を作成し、行を足して正しく変わるか検算できる。</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>開始日の式をAIに作らせる。
-行を足して結果が正しく変わるか確かめる。</t>
+          <t>延長・停止開始日（3回目の翌日）の式をGeminiに作らせる。
+自分で行を足し、結果が正しく変わるか確かめる。</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -2371,19 +2369,19 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>メールで納品する
+          <t>Gmailで納品する
 基本教材 3章3</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>集計の結果をメールに正しく書き、納品できる。</t>
+          <t>Geminiで納品メールを下書きし、集計の結果を本文に入れてGmailで送信できる。</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>スライド3枚、画像から物を消す。
-Gemini で下書きし、Gmail で送る。
+          <t>Googleスライド3枚。画像から物を消す。
+Geminiで納品メールを下書きし、Gmailで送る（件名の約束）。
 成果物3の通し練習（50分）。</t>
         </is>
       </c>
@@ -2412,12 +2410,12 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>成果物3　メールで納品する（実技）</t>
+          <t>成果物3　面接練習室の張り紙一式と納品メール（実技）</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>誤り一覧・集計表・画像3枚をそろえ、メールで納品できる。</t>
+          <t>下書きの誤り9件を直し、張り紙・スライド3枚・集計表・誤り一覧・画像3枚をGmailで納品できる。</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -2427,7 +2425,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>成果物3（クラスルーム）</t>
+          <t>成果物3</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
@@ -2442,7 +2440,7 @@
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>受付はクラスルームで設定。本人の証拠は合言葉と作成時刻</t>
+          <t>受付はクラスルームで設定</t>
         </is>
       </c>
     </row>
@@ -2460,13 +2458,14 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>書かれていないこと・重複・詰め込みを直せる。</t>
+          <t>AIが作った詰め込みすぎのGoogleスライドを、GeminiのCanvasで1枚1つの話に作り直せる。</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
           <t>成果物3の答え合わせ。
-Canvas で1枚1つの話に作り直す。</t>
+元のスライドを原文と照合し、脱落・重複を直す。
+Canvasで作り直し、同じ頼み方で2枚を再現する。</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -2500,13 +2499,14 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>集計・グラフ・報告の数字をそろえ、説明会に招待できる。</t>
+          <t>月で数え直す集計表とグラフを作成し、Google Meet付きの予定をGoogleカレンダーで作って招待できる。</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>月で数え直す式とグラフをAIと作る。画像に文字を入れる。
-カレンダーに Meet つきの予定を作り招待する。</t>
+          <t>月で数え直す式と部屋別件数のグラフ。画像に文字を入れる。
+Geminiの連携アプリでGoogleカレンダー・Keepに予定を入れる。
+Meetを付けて教員を招待する。</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -2538,12 +2538,12 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>成果物4　最終課題に近い一連の仕事（実技）</t>
+          <t>成果物4　撮影ブースの説明会の準備一式（実技）</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>スライド・集計表・画像3枚・納品メール・招待を提出できる。</t>
+          <t>元のスライド8枚を作り直し、集計表・画像3枚・納品メール・Google Meet付きの招待を作成して提出できる。</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>成果物4（クラスルーム）</t>
+          <t>成果物4</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
@@ -2568,7 +2568,7 @@
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>受付はクラスルームで設定。本人の証拠は合言葉と作成時刻</t>
+          <t>受付はクラスルームで設定</t>
         </is>
       </c>
     </row>
@@ -2586,13 +2586,14 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>期間で条件が変わる集計と誤り一覧を作れる。</t>
+          <t>期間で上限が変わる式を作成し、Gemini Notebookで条番号つきの誤り一覧を作れる。</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
           <t>成果物4の答え合わせ。
-Flash と Pro の使い分け。</t>
+FlashとProの使い分け（速さと正確さ）。
+条番号つきの誤り一覧、期間で上限が変わる式。</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -2626,12 +2627,12 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>4つを時間内に仕上げ、画面録画つきで提出できる。</t>
+          <t>最終課題の練習版を画面録画しながら60分で仕上げ、Googleフォームで提出できる。</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>ガイド付き学習で自分の誤りを振り返る。
+          <t>Geminiの学習モードで自分の誤りを振り返る。
 最終課題の通し練習（60分、画面録画）。</t>
         </is>
       </c>
@@ -2660,22 +2661,22 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>成果物5　4つを誤りゼロで仕上げる（実技）</t>
+          <t>成果物5（最終課題）　充電ロッカーの張り紙一式（実技）</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>原文だけを正として4つを誤りなく仕上げられる。</t>
+          <t>原文だけを正として、張り紙・スライド3枚・集計表と誤り一覧・画像3枚を作成して提出できる。</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>説明10分、個人作業90分。スマホ・AI使用可。作業中は画面録画。</t>
+          <t>説明10分、個人作業90分。スマホ・AI使用可。</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>成果物5（クラスルーム）</t>
+          <t>成果物5</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
@@ -2690,7 +2691,7 @@
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
-          <t>受付はクラスルームで設定。本人の証拠は合言葉と画面録画（リンクは次の授業の開始まで）</t>
+          <t>受付はクラスルームで設定。作業中は画面録画（リンクは次の授業の開始まで）</t>
         </is>
       </c>
     </row>
@@ -2853,10 +2854,10 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>仕事のルール・メール・申込データを日本語で読み、連絡と記録を正しく行う。
-架空の学内講座の運営を一人（成果物2は2人1組）で行い、回ごとに材料と条件が増える。
-扱うのはメールの宛先、共有の設定、個人情報・著作権、データの数え方。わからない時はAIで自分で解決し、ルールと照らして確かめる。
-マーケティング・AI演習（実践）につながり、この科目は「運用する力」を担う。</t>
+          <t>架空の学内講座の運営を、前任者から引き継いだ設定で進める。
+届いたメール・運営のルール・申込データを読み、Gmailで日程確定や補欠のお知らせを送り、Google Meetで運営会議を開いて議事録とToDoを作る。
+Googleドライブの共有フォルダを整理して共有設定を直し、スプレッドシートで申込を数えて確定・補欠・費用を出す。成果物は5回（成果物2は2人1組）で、画面録画などを添えてGoogleフォームで提出する。
+わからない時はGeminiで自分で解決し、答えは運営のルールと照らして確かめる。</t>
         </is>
       </c>
       <c r="B6" s="2" t="n"/>
@@ -2864,11 +2865,10 @@
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>教科書：『留学生のためのITリテラシー』（参考。対応ページを授業計画に示す）
+          <t>教科書：『留学生のためのITリテラシー』（対応ページを授業計画に示す）
 基本教材：Geminiビジネス活用ガイド（最新の機能で扱う）
-配布：運営のルール、メール、申込データ、前任者の下書き
-環境：スマホ、個人の Google アカウント（無料）
-ツール：Gemini、Gemini Notebook、Gmail、カレンダー、Meet、Keep、ドキュメント、ドライブ、スプレッドシート、フォーム、フォト、YouTube、画面録画、Classroom</t>
+環境：スマホ、個人の Google アカウント（無料）。配布：運営のルール、メール、申込データ、前任者の下書き
+ツール：Gemini、Gemini Notebook、Gmail、Googleカレンダー、Google Meet、Keep、Googleドキュメント、Googleドライブ、スプレッドシート、Googleフォーム、Googleフォト、YouTube、画面録画</t>
         </is>
       </c>
       <c r="F6" s="2" t="n"/>
@@ -2936,10 +2936,10 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>1. メールから最新の決定を拾い、下書きの誤りだけを直して、正しい宛先（BCC など）で送れる。
-2. 会議を開き、議事録と ToDo の期限をルールどおりに作れる。
-3. 共有フォルダを整理し、共有の設定を安全に直せる。
-4. AIに作らせた式の結果を確かめ、申込を数えて確定と補欠を決められる。</t>
+          <t>1. メールから最新の決定を拾い、下書きの誤りだけを直して、GmailでBCCなど正しい宛先で送れる。
+2. Google Meetで会議を開き、Googleドキュメントで議事録を作成し、ToDoの期限をGoogleカレンダーに入れられる。
+3. Googleドライブの共有フォルダを整理し、共有設定（リンク公開、閲覧者・編集者）を安全に直せる。
+4. Geminiが作った式をスプレッドシートで検算し、申込を数えて確定・補欠と費用を出せる。</t>
         </is>
       </c>
       <c r="B12" s="2" t="n"/>
@@ -2948,13 +2948,8 @@
       <c r="E12" s="5" t="inlineStr">
         <is>
           <t>採点基準は学校規定に準ずる。
-【独自の基準】
-・成果物は、課題ごとに示した条件を1つずつ○✖で見て、○の分だけ点を足す。1か所まちがえても、ほかの点は失わない。
-・本人が作った証拠（合言葉・画面録画・版の履歴など）が無い提出は0点。
-・材料の数字は学生ごとに違う。他人の答えを写しても点にならない。
-・作業時間は目安で、採点しない。受付時間はクラスルームで課題ごとに設定する。
-・小テストは満点で○。点＝20×○の数÷14（成果物の回は行わない）。欠席は✖。
-・出席率70%の学生でも、成果物で48点取ればD（60点）に届く設計にしている。</t>
+成果物は、課題ごとの条件を満たした分だけ点を足す。
+本人が作った証拠（録画など）の無い提出は0点。</t>
         </is>
       </c>
       <c r="F12" s="2" t="n"/>
@@ -3022,8 +3017,8 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>成果物 80点（8・12・15・20・25点）
-小テスト 20点（成果物の回を除く14回。授業中のみ、満点まで再提出可）</t>
+          <t>成果物 80点（5回：8・12・15・20・25点）
+小テスト 20点（成果物の回以外の毎回）</t>
         </is>
       </c>
       <c r="B18" s="2" t="n"/>
@@ -3031,8 +3026,8 @@
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>小テスト：その場で結果を返し、満点まで再提出できる。
-成果物：前の回に別の番号の材料で通し練習（14・18回は自己採点も）。成果物1は本番の回で答え合わせ。採点の後に振り返る。</t>
+          <t>小テストはその場で返し、満点まで出し直せる。
+成果物は前の回に練習し、本番の後に答え合わせをする。</t>
         </is>
       </c>
       <c r="F18" s="2" t="n"/>
@@ -3149,19 +3144,19 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>To・CC・BCC を使い分けて送り、曜日を確かめられる。</t>
+          <t>GmailでTo・CC・BCCを使い分けてメールを送り、Googleカレンダーで日付の曜日を確かめられる。</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>科目の進め方と評価。
-Gmail の To・CC・BCC、カレンダーで曜日の確認。
-提出フォームの練習。</t>
+          <t>科目の進め方と評価。Geminiの基本操作。
+GmailのTo・CC・BCC、Googleカレンダーで曜日の確認。
+Googleフォームで提出の練習。</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>練習の提出</t>
+          <t>提出の練習</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
@@ -3190,12 +3185,12 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>最新の合意を拾い、正しい宛先で確定のメールを送れる。</t>
+          <t>メールのやり取りから最新の日時・会場を拾い、Geminiが作った返信の下書きを直してGmailで送れる。</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>AIに返信の下書きを作らせ、決まりと照らして直す。
+          <t>Geminiに返信の下書きを作らせ、運営のルールと照らして直す。
 成果物1の通し練習（別の番号の材料）。</t>
         </is>
       </c>
@@ -3224,12 +3219,12 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>成果物1　日程変更への返信（実技）</t>
+          <t>成果物1　日程確定のメール（実技）</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>最新の日時・会場を拾い、BCC で確定のメールを送れる。</t>
+          <t>4通のメールから最新の日時・会場を拾って曜日を確かめ、GmailのBCCで日程確定のメールを送り、Googleフォームで提出できる。</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -3239,7 +3234,7 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>成果物1（提出フォーム）</t>
+          <t>成果物1</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -3254,7 +3249,7 @@
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>受付はクラスルームで設定。証拠はメールの差出人と提出フォームのアドレスの照合</t>
+          <t>受付はクラスルームで設定</t>
         </is>
       </c>
     </row>
@@ -3272,13 +3267,13 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>カレンダーから招待して Meet を開き、チャットで話し合える。</t>
+          <t>GoogleカレンダーからGoogle Meetの会議に招待し、チャットで話し合ってKeepのチェックリストで分担できる。</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>カレンダーから招待し、Meet のチャットで話す。
-Keep のチェックリストで分担。Gemini の履歴と名前の変更。</t>
+          <t>GoogleカレンダーからMeetに招待し、Meetのチャットで話す。
+Keepのチェックリストで分担。Geminiのチャット履歴と名前の変更。</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -3306,19 +3301,19 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>議事録と ToDo の期限
+          <t>議事録とToDoの期限
 基本教材 第3章3／教科書 p.88〜91・104〜107</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>議事録を作り、ToDo の期限を決まりどおりに出せる。</t>
+          <t>Googleドキュメントで議事録を作成し、ToDoの期限を決まり（営業日・曜日）どおりに計算できる。</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>AIで議事録の型を作り、話していないことが足されていないか確かめる。
-期限の計算（営業日・曜日）。</t>
+          <t>Geminiで議事録の型を作り、話していないことが足されていないか確かめる。
+ToDoの期限の計算（営業日・曜日）。</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -3352,12 +3347,12 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>議事録の要点を出させ、元と照らして確かめられる。</t>
+          <t>Gemini Notebookに議事録を入れて要点を出させ、元の議事録と照らして確かめられる。</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Gemini Notebook で議事録の要点を出させ、元と照らす。
+          <t>Gemini Notebookで議事録の要点を出させ、元と照らす。
 成果物2の通し練習（2人1組、短い版）。</t>
         </is>
       </c>
@@ -3386,23 +3381,22 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>成果物2　運営会議（実技・2人1組）</t>
+          <t>成果物2　運営会議の議事録とToDo（実技・2人1組）</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>会議を開き、議事録を正しい宛先で送り、ToDo を期限どおりに入れられる。</t>
+          <t>Google Meetで会議を開き、Googleドキュメントの議事録をGmailで相手に送り、ToDoの期限をGoogleカレンダーに入れて提出できる。</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>説明10分、2人1組で作業し開始から85分を目安に提出。スマホ・AI使用可。
-会議は Meet のチャットで2回（各15分）。</t>
+          <t>説明10分、2人1組で作業85分（Meetのチャットで会議2回、各15分）。スマホ・AI使用可。</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>成果物2（提出フォーム）</t>
+          <t>成果物2</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -3417,7 +3411,7 @@
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>受付はクラスルームで設定。証拠は合言葉と版の履歴。奇数の時は1組だけ3人</t>
+          <t>受付はクラスルームで設定。奇数の時は1組だけ3人</t>
         </is>
       </c>
     </row>
@@ -3435,12 +3429,12 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>中身の日付で最新版を見分け、決まりどおりに整理できる。</t>
+          <t>Googleドライブで中身の日付から最新版を見分け、名前の変更・フォルダ作成・移動で決まりどおりに整理できる。</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>ドライブで名前の変更・フォルダ作成・移動。
+          <t>Googleドライブで名前の変更・フォルダ作成・移動。
 中身の日付で最新版を見分ける。</t>
         </is>
       </c>
@@ -3475,14 +3469,14 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>リンク公開を止め、閲覧者・編集者を正しく設定できる。</t>
+          <t>Googleドライブのリンク公開を止めて閲覧者・編集者を正しく設定し、Googleフォトのアルバムを必要な人だけに共有できる。</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>AIに写り込みと撮影場所の確かめ方を聞く。
-共有の設定（リンク公開、閲覧者・編集者、学外への名簿）。
-フォトのアルバムと切り取り。</t>
+          <t>Geminiに写り込みと撮影場所の確かめ方を聞く。
+共有設定（リンク公開、閲覧者・編集者、学外への名簿）。
+Googleフォトのアルバムと切り取り。</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -3516,13 +3510,13 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>空白・取消・申し込み直し・締切後を正しく扱い、人数を出せる。</t>
+          <t>Geminiが作った式でスプレッドシートの申込を数え（空白・取消・申し込み直し・締切後）、3つの方法で検算できる。</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>AIに式を作らせて貼る。
-検算：①答えのわかる小さな表で試す ②範囲をなぞり画面下の合計・個数と比べる ③見当と比べる。
+          <t>Geminiに式を作らせてスプレッドシートに貼る。
+検算：答えのわかる小さな表で試す／範囲をなぞり画面下の合計・個数と比べる／見当と比べる。
 画面録画をして成果物3の通し練習。</t>
         </is>
       </c>
@@ -3556,7 +3550,7 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>フォルダを整理して危ない共有を止め、人数をメールで報告できる。</t>
+          <t>Googleドライブの共有フォルダを整理して危ない共有を止め、スプレッドシートで出した人数をGmailで報告し、画面録画を添えて提出できる。</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
@@ -3566,7 +3560,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>成果物3（提出フォーム）</t>
+          <t>成果物3</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
@@ -3581,7 +3575,7 @@
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>受付はクラスルームで設定。証拠は合言葉と録画。録画は次の授業の開始まで可</t>
+          <t>受付はクラスルームで設定。録画は次の授業の開始まで可</t>
         </is>
       </c>
     </row>
@@ -3599,12 +3593,12 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>最新の回答だけを残し、定員で確定と補欠に分けられる。</t>
+          <t>スプレッドシートで最新の回答だけを残して時刻順に並べ、定員で確定と補欠に分けられる。</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>AIに式を作らせ、最新の回答だけを残して時刻順に並べる。
+          <t>Geminiに式を作らせ、最新の回答だけを残して時刻順に並べる。
 定員を超えた人を補欠にする。</t>
         </is>
       </c>
@@ -3639,12 +3633,12 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>下書きの誤りだけを直し、データを変えても式が正しいか確かめられる。</t>
+          <t>Googleドキュメントの下書きの誤りだけを直し、データを差し替えても式の結果が正しいか確かめられる。</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>AIの直しを決まりと照らして選ぶ（直しすぎない）。
+          <t>Geminiの直しを運営のルールと照らして選ぶ（直しすぎない）。
 データを差し替えて式の結果を確かめる。</t>
         </is>
       </c>
@@ -3679,13 +3673,13 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>通し練習をして、採点の表で自分の誤りを見つけられる。</t>
+          <t>成果物4の通し練習を40分で行い、採点表で自己採点して自分の誤りを見つけられる。</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
           <t>成果物4の通し練習（40分）と自己採点。
-ガイド付き学習で誤りを振り返る。</t>
+Geminiのガイド付き学習で誤りを振り返る。</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -3713,12 +3707,12 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>成果物4　補欠の決定とお知らせ（実技）</t>
+          <t>成果物4　補欠の決定とお知らせメール（実技）</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>補欠を決め、下書きを直して補欠の方に BCC で予約送信できる。</t>
+          <t>申込データから確定と補欠を決め、下書きを直したお知らせをGmailのBCCで予約送信し、画面録画を添えて提出できる。</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
@@ -3728,7 +3722,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>成果物4（提出フォーム）</t>
+          <t>成果物4</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
@@ -3743,7 +3737,7 @@
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>受付はクラスルームで設定。証拠は合言葉と録画（YouTube 限定公開）。録画は次の授業の開始まで可</t>
+          <t>受付はクラスルームで設定。録画はYouTube限定公開、次の授業の開始まで可</t>
         </is>
       </c>
     </row>
@@ -3761,12 +3755,12 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>改定後のルールで、表記ゆれをそろえて数えられる。</t>
+          <t>Gemini Notebookで改定後のルールを確かめ、表記ゆれ（全角・古い選択肢）をそろえて申込を数えられる。</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Gemini Notebook にルールを入れ、根拠つきで答えさせる。
+          <t>Gemini Notebookにルールを入れ、根拠つきで答えさせる。
 表記ゆれ（全角・古い選択肢）をそろえて数える。</t>
         </is>
       </c>
@@ -3801,7 +3795,7 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>録画・画像・名簿を決まりどおりに扱い、費用を計算できる。</t>
+          <t>録画・画像・名簿を決まりどおりに扱う文面に直し、印刷費（確定者＋予備）を計算できる。</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
@@ -3845,12 +3839,12 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>予行をして、採点の表で自己採点できる。</t>
+          <t>最終課題の予行を別の番号の材料で40分行い、自己採点できる。</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Flash（速い）と Pro（深い）の使い分け。
+          <t>GeminiのFlash（速い）とPro（深い）の使い分け。
 最終課題の予行（別の番号で40分）と自己採点。</t>
         </is>
       </c>
@@ -3879,12 +3873,12 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>成果物5　講座運用の引き継ぎ（実技・最終課題）</t>
+          <t>成果物5　講座運営の引き継ぎ（実技・最終課題）</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>人数と費用を出し、誤りだけ直したメールを安全な共有で仕上げられる。</t>
+          <t>申込データから人数と印刷費を出し、前任者のメールの誤りだけを直して安全な共有設定で仕上げ、画面録画を添えて提出できる。</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
@@ -3894,7 +3888,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>成果物5（提出フォーム）</t>
+          <t>成果物5</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
@@ -3909,7 +3903,7 @@
       </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
-          <t>受付はクラスルームで設定。証拠は合言葉と録画</t>
+          <t>受付はクラスルームで設定</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Unify course overview and goals across three syllabi
Overview becomes one sentence; goals become five items, one per
deliverable, in the form 'Xを使ってYがZできる'. Also repair the
handover header that the previous entry had been spliced into.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014qy3US5uqWgiaAnx8zBN8m
</commit_message>
<xml_diff>
--- a/docs/drafts/syllabus-sheets/syllabus.xlsx
+++ b/docs/drafts/syllabus-sheets/syllabus.xlsx
@@ -586,10 +586,7 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>架空の「日本語カフェ」から「もっと留学生に来てほしい」と頼まれた設定で進める。
-Googleフォームでアンケートを作り、回答をスプレッドシートで集計し、その数字で「誰に・何を・いつ・どこで」告知するかを決める。
-決めた内容で、SNS用のカルーセル（Canvaで作る数ページの画像。MP4で提出）と投稿文を作る。実際には公開しない。
-わからない時はGeminiで自分で解決し、出てきた答えや式は必ず確かめる。</t>
+          <t>マーケティング手法をビジネスで活用するための基礎を養成する科目。</t>
         </is>
       </c>
       <c r="B6" s="2" t="n"/>
@@ -668,10 +665,11 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>1. 目的に合う形式でGoogleフォームのアンケートを作れる。
-2. 回答をスプレッドシートで正しく集計できる（Geminiが作った式を検算する）。
-3. 集計結果から、ターゲット・内容・日時・投稿先を決められる。
-4. 決めた内容どおりのカルーセルと投稿文を作れる。</t>
+          <t>1. Googleフォームとスプレッドシートを使って、アンケートの集計結果から告知スライドが作成できる。
+2. GeminiとCanvaを使って、集計した数字を載せたカルーセル動画が作成できる。
+3. Googleマップと画像生成を使って、ターゲットと競合を踏まえたカルーセル動画が作成できる。
+4. GoogleトレンドとGA4を使って、投稿先と日時を決めたカルーセル動画と投稿文が作成できる。
+5. アンケートの集計結果を使って、「誰に・何を・いつ・どこで」を決めたカルーセル動画と投稿文が作成できる。</t>
         </is>
       </c>
       <c r="B12" s="2" t="n"/>
@@ -1676,10 +1674,7 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>架空の学校の図書室や事務室から「利用ルールの張り紙を作り、利用記録を集計してほしい」と頼まれた設定で進める。
-先輩がAIで作った下書きをルールの原文だけを正として直し、張り紙（Googleドキュメント）・Googleスライド・集計表（スプレッドシート）・画像の4つを作る。
-作ったものは共有設定とGoogleフォームで提出する。回が進むとGmailでの納品やGoogleカレンダーの招待が加わる。
-わからない時はGeminiで自分で解決し、出てきた答えや式は必ず確かめる。</t>
+          <t>生成AIをビジネスで活用するための基礎を養成する科目。</t>
         </is>
       </c>
       <c r="B6" s="2" t="n"/>
@@ -1758,10 +1753,11 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>1. ルールの原文だけを正として、AIの下書きの誤りを直した張り紙と誤り一覧を作成できる。
-2. Geminiに作らせた式を検算し、行を足しても正しく動く集計表をスプレッドシートで作成できる。
-3. 条件を守った画像を3枚そろえ、約束どおりの形のGoogleスライドを作成できる。
-4. 作ったものを共有設定・Gmail・Googleカレンダーの招待で届けられる。</t>
+          <t>1. Geminiとドキュメント・スプレッドシートを使って、張り紙・スライド・集計表・画像の一式が作成できる。
+2. Gemini Notebookを使って、下書きの誤りを直した張り紙と、画像3枚をそろえたスライドが作成できる。
+3. Gmailを使って、誤り一覧を添えた張り紙一式が納品できる。
+4. GmailとGoogleカレンダーを使って、説明会のスライド・納品メール・Google Meet付きの招待が作成できる。
+5. Geminiを使って、原文だけを正とした張り紙・スライド・集計表・画像の一式が作成できる。</t>
         </is>
       </c>
       <c r="B12" s="2" t="n"/>
@@ -2854,10 +2850,7 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>架空の学内講座の運営を、前任者から引き継いだ設定で進める。
-届いたメール・運営のルール・申込データを読み、Gmailで日程確定や補欠のお知らせを送り、Google Meetで運営会議を開いて議事録とToDoを作る。
-Googleドライブの共有フォルダを整理して共有設定を直し、スプレッドシートで申込を数えて確定・補欠・費用を出す。成果物は5回（成果物2は2人1組）で、画面録画などを添えてGoogleフォームで提出する。
-わからない時はGeminiで自分で解決し、答えは運営のルールと照らして確かめる。</t>
+          <t>ITツールをビジネスで活用するための基礎を養成する科目。</t>
         </is>
       </c>
       <c r="B6" s="2" t="n"/>
@@ -2936,10 +2929,11 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>1. メールから最新の決定を拾い、下書きの誤りだけを直して、GmailでBCCなど正しい宛先で送れる。
-2. Google Meetで会議を開き、Googleドキュメントで議事録を作成し、ToDoの期限をGoogleカレンダーに入れられる。
-3. Googleドライブの共有フォルダを整理し、共有設定（リンク公開、閲覧者・編集者）を安全に直せる。
-4. Geminiが作った式をスプレッドシートで検算し、申込を数えて確定・補欠と費用を出せる。</t>
+          <t>1. Gmailを使って、複数のメールから拾った最新の日時・会場で日程確定のメールが送信できる。
+2. Google MeetとGoogleカレンダーを使って、会議の議事録作成とToDoの期限登録ができる。
+3. Googleドライブとスプレッドシートを使って、共有フォルダの整理と人数の報告ができる。
+4. スプレッドシートとGmailを使って、確定・補欠の決定とお知らせメールの予約送信ができる。
+5. スプレッドシートとGoogleドライブを使って、人数・印刷費の算出と安全な共有設定での引き継ぎができる。</t>
         </is>
       </c>
       <c r="B12" s="2" t="n"/>

</xml_diff>